<commit_message>
feat: register Hand-Taiyin Shidong disorder clinical matrix report (KO/EN) and update portal index
</commit_message>
<xml_diff>
--- a/04_번역원고_및_임상매트릭스/영추경맥_수태음시동병_매트릭스/영추경맥_수태음시동병_해부임상_매트릭스.xlsx
+++ b/04_번역원고_및_임상매트릭스/영추경맥_수태음시동병_매트릭스/영추경맥_수태음시동병_해부임상_매트릭스.xlsx
@@ -731,7 +731,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{"A1_수태음본경_아래팔": ["Cephalic vein", "Radial artery", "Radial vein", "Brachioradialis", "Pronator quadratus", "Flexor digitorum superficialis", "Set of dorsal digital veins"], "A2_앞가슴벽": ["External intercostal muscle", "Internal intercostal muscle", "Internal thoracic vein", "Internal thoracic artery", "Transversus thoracis", "Pectoralis minor", "Lateral thoracic artery"], "B2_목앞_빗장위": ["Common carotid artery", "Internal thoracic vein", "Sternohyoid", "Omohyoid", "Sternocleidomastoid", "Platysma"], "B1_등_흉추옆": ["Transverse cervical artery", "Splenius cervicis", "Longissimus", "Rhomboid major"]}</t>
+          <t>{"A1_상지": ["Cephalic vein", "Radial artery", "Radial vein", "Brachioradialis", "Pronator quadratus", "Flexor digitorum superficialis", "Set of dorsal digital veins"], "A2a_앞가슴벽": ["External intercostal muscle", "Internal intercostal muscle", "Internal thoracic vein", "Internal thoracic artery", "Transversus thoracis", "Pectoralis minor", "Lateral thoracic artery"], "B2_목앞_빗장위": ["Common carotid artery", "Internal thoracic vein", "Sternohyoid", "Omohyoid", "Sternocleidomastoid", "Platysma"], "B1_등_흉추옆": ["Transverse cervical artery", "Splenius cervicis", "Longissimus", "Rhomboid major"]}</t>
         </is>
       </c>
     </row>
@@ -19945,9 +19945,9 @@
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19968,7 +19968,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>대분류(5군)</t>
+          <t>대분류(8군)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -19978,7 +19978,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>소분류 번호(16군)</t>
+          <t>소분류(16군)</t>
         </is>
       </c>
     </row>
@@ -20000,7 +20000,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>B1 등 흉추 옆·어깨 위</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -20008,8 +20008,10 @@
           <t>B1 등 흉추 옆·어깨 위</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>3</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>B1 등 흉추 옆·어깨 위</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -20030,7 +20032,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>B1 등 흉추 옆·어깨 위</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -20038,8 +20040,10 @@
           <t>B1 등 흉추 옆·어깨 위</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>3</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>B1 등 흉추 옆·어깨 위</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -20060,16 +20064,18 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>D2 C7 극돌기(大椎)</t>
+          <t>D 명치(鳩尾)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>A4 명치(鳩尾)</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>16</v>
+          <t>D 명치(鳩尾)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>D 명치(鳩尾)</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -20090,16 +20096,18 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>D1 흉골 정중(玉堂)</t>
+          <t>D 흉골 정중(玉堂)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>D1 흉골 정중(玉堂)</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>15</v>
+          <t>D 흉골 정중(玉堂)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>D 흉골 정중(玉堂)</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -20120,7 +20128,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>B2 목 앞·빗장위</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -20128,8 +20136,10 @@
           <t>B2a 흉골위패임·흉골자루</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>4</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>B2a 흉골위패임·흉골자루</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -20158,8 +20168,10 @@
           <t>C 하지 원위</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>1</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>C1 발등(足臨泣)</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -20180,16 +20192,18 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>A1 수태음 본경·손목 자쪽</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>6</v>
+          <t>A1 상지(수태음 본경·손목·손가락)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>A1b 손목 자쪽(陰郄·神門)</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -20210,16 +20224,18 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>A2 앞가슴벽</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>9</v>
+          <t>A2 앞가슴벽(늑간·가슴근신경)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>A2a 앞가슴벽 2~5늑간</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -20240,16 +20256,18 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>A2 앞가슴벽</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>10</v>
+          <t>A2 앞가슴벽(늑간·가슴근신경)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>A2b 빗장 아래(俞府)</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -20270,16 +20288,18 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>A1 수태음 본경·손목 자쪽</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>7</v>
+          <t>A1 상지(수태음 본경·손목·손가락)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>A1c 손가락(少商·三間·前谷·商陽)</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -20300,16 +20320,18 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>D2 C7 극돌기(大椎)</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>11</v>
+          <t>A2c 앞가슴벽 바깥(中府)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>A2c 앞가슴벽 바깥(中府)</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -20330,16 +20352,18 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>A1 수태음 본경·손목 자쪽</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>7</v>
+          <t>A1 상지(수태음 본경·손목·손가락)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>A1c 손가락(少商·三間·前谷·商陽)</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -20360,16 +20384,18 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>A1 수태음 본경·손목 자쪽</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>8</v>
+          <t>A1 상지(수태음 본경·손목·손가락)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>A1a 수태음 본경 사슬(天府~太淵)</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -20390,16 +20416,18 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>A1 수태음 본경·손목 자쪽</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
-        <v>8</v>
+          <t>A1 상지(수태음 본경·손목·손가락)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>A1a 수태음 본경 사슬(天府~太淵)</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -20420,16 +20448,18 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>A1 수태음 본경·손목 자쪽</t>
-        </is>
-      </c>
-      <c r="F16" t="n">
-        <v>8</v>
+          <t>A1 상지(수태음 본경·손목·손가락)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>A1a 수태음 본경 사슬(天府~太淵)</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -20450,16 +20480,18 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>A2 앞가슴벽</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>9</v>
+          <t>A2 앞가슴벽(늑간·가슴근신경)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>A2a 앞가슴벽 2~5늑간</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -20480,16 +20512,18 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>A1 수태음 본경·손목 자쪽</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>7</v>
+          <t>A1 상지(수태음 본경·손목·손가락)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>A1c 손가락(少商·三間·前谷·商陽)</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -20510,16 +20544,18 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>A2 앞가슴벽</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>9</v>
+          <t>A2 앞가슴벽(늑간·가슴근신경)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>A2a 앞가슴벽 2~5늑간</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -20540,7 +20576,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>B2 목 앞·빗장위</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -20548,8 +20584,10 @@
           <t>B2b 목 앞·빗장위</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>5</v>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>B2b 목 앞·빗장위</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -20570,7 +20608,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>B2 목 앞·빗장위</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -20578,8 +20616,10 @@
           <t>B2b 목 앞·빗장위</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>5</v>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>B2b 목 앞·빗장위</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -20600,7 +20640,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>B2 목 앞·빗장위</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -20608,8 +20648,10 @@
           <t>B2a 흉골위패임·흉골자루</t>
         </is>
       </c>
-      <c r="F22" t="n">
-        <v>4</v>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>B2a 흉골위패임·흉골자루</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -20630,16 +20672,18 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>D2 C7 극돌기(大椎)</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>12</v>
+          <t>A2d 옆가슴(輒筋)</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>A2d 옆가슴(輒筋)</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -20660,16 +20704,18 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>A1 수태음 본경·손목 자쪽</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>6</v>
+          <t>A1 상지(수태음 본경·손목·손가락)</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>A1b 손목 자쪽(陰郄·神門)</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -20690,16 +20736,18 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>A2 앞가슴벽</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>9</v>
+          <t>A2 앞가슴벽(늑간·가슴근신경)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>A2a 앞가슴벽 2~5늑간</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -20720,16 +20768,18 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>A2 앞가슴벽</t>
-        </is>
-      </c>
-      <c r="F26" t="n">
-        <v>9</v>
+          <t>A2 앞가슴벽(늑간·가슴근신경)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>A2a 앞가슴벽 2~5늑간</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -20758,8 +20808,10 @@
           <t>C 하지 원위</t>
         </is>
       </c>
-      <c r="F27" t="n">
-        <v>2</v>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>C2 발목 안쪽(大鐘)</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -20780,16 +20832,18 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>D 갈비활(期門)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>A5 갈비활(期門)</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>13</v>
+          <t>D 갈비활(期門)</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>D 갈비활(期門)</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -20810,16 +20864,18 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>A1 수태음 본경·손목 자쪽</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
-        <v>8</v>
+          <t>A1 상지(수태음 본경·손목·손가락)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>A1a 수태음 본경 사슬(天府~太淵)</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -20840,16 +20896,18 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>A1 수태음 본경·손목 자쪽</t>
-        </is>
-      </c>
-      <c r="F30" t="n">
-        <v>8</v>
+          <t>A1 상지(수태음 본경·손목·손가락)</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>A1a 수태음 본경 사슬(天府~太淵)</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -20870,16 +20928,18 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>A1 수태음 본경·손목 자쪽</t>
-        </is>
-      </c>
-      <c r="F31" t="n">
-        <v>8</v>
+          <t>A1 상지(수태음 본경·손목·손가락)</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>A1a 수태음 본경 사슬(天府~太淵)</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -20900,16 +20960,18 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>A1 수태음 본경·손목 자쪽</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>8</v>
+          <t>A1 상지(수태음 본경·손목·손가락)</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>A1a 수태음 본경 사슬(天府~太淵)</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -20930,7 +20992,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>B1 등 흉추 옆·어깨 위</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -20938,8 +21000,10 @@
           <t>B1 등 흉추 옆·어깨 위</t>
         </is>
       </c>
-      <c r="F33" t="n">
-        <v>3</v>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>B1 등 흉추 옆·어깨 위</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -20960,7 +21024,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>B1 등 흉추 옆·어깨 위</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -20968,8 +21032,10 @@
           <t>B1 등 흉추 옆·어깨 위</t>
         </is>
       </c>
-      <c r="F34" t="n">
-        <v>3</v>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>B1 등 흉추 옆·어깨 위</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -20990,16 +21056,18 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>D2 C7 극돌기(大椎)</t>
+          <t>D C7 극돌기(大椎)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>D2 C7 극돌기(大椎)</t>
-        </is>
-      </c>
-      <c r="F35" t="n">
-        <v>14</v>
+          <t>D C7 극돌기(大椎)</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>D C7 극돌기(大椎)</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -21020,16 +21088,18 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>A2 앞가슴벽</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>9</v>
+          <t>A2 앞가슴벽(늑간·가슴근신경)</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>A2a 앞가슴벽 2~5늑간</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -21050,16 +21120,18 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>A1 수태음 본경·손목 자쪽</t>
-        </is>
-      </c>
-      <c r="F37" t="n">
-        <v>7</v>
+          <t>A1 상지(수태음 본경·손목·손가락)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>A1c 손가락(少商·三間·前谷·商陽)</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -21080,16 +21152,18 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>A2 앞가슴벽</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>9</v>
+          <t>A2 앞가슴벽(늑간·가슴근신경)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>A2a 앞가슴벽 2~5늑간</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -21110,16 +21184,18 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>A 팔신경얼기 영역</t>
+          <t>A 팔신경얼기 영역(상지·앞가슴벽)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>A2 앞가슴벽</t>
-        </is>
-      </c>
-      <c r="F39" t="n">
-        <v>9</v>
+          <t>A2 앞가슴벽(늑간·가슴근신경)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>A2a 앞가슴벽 2~5늑간</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -23259,7 +23335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -23275,7 +23351,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>중분류</t>
+          <t>소분류</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -23317,121 +23393,117 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C 하지 원위</t>
+          <t>C1 발등(足臨泣)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GB41, KI4</t>
+          <t>GB41</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>0/1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>0/1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>0/1</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0/2</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>0.301</v>
-      </c>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>B1 등 흉추 옆·어깨 위</t>
+          <t>C2 발목 안쪽(大鐘)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BL13, BL17, BL14, GB21</t>
+          <t>KI4</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>0/1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1/4</t>
+          <t>0/1</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>4/4</t>
+          <t>0/1</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0/4</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>0.525</v>
-      </c>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>B2a 흉골위패임·흉골자루</t>
+          <t>B1 등 흉추 옆·어깨 위</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CV22, CV21</t>
+          <t>BL13, BL17, BL14, GB21</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2/2</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2/2</t>
+          <t>1/4</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2/2</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>0/4</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0.571</v>
+        <v>0.525</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>B2b 목 앞·빗장위</t>
+          <t>B2a 흉골위패임·흉골자루</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -23439,17 +23511,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ST12, ST9</t>
+          <t>CV22, CV21</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -23459,201 +23531,207 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>0/2</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.399</v>
+        <v>0.571</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>A1 수태음 본경·손목 자쪽</t>
+          <t>B2b 목 앞·빗장위</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>HT7, LI3, LU11, LU5, LU7, LU9, SI2, HT6, LU3, LU4, LU6, LU8, LI1</t>
+          <t>ST12, ST9</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>13/13</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13/13</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0/13</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0/13</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.418</v>
+        <v>0.399</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>A2 앞가슴벽</t>
+          <t>A1b 손목 자쪽(陰郄·神門)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>KI25, KI27, PC1, SP18, KI22, KI23, KI24, ST16, ST18</t>
+          <t>HT7, HT6</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>9/9</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9/9</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1/9</t>
+          <t>0/2</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0/9</t>
+          <t>0/2</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0.493</v>
+        <v>0.863</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>D2 C7 극돌기(大椎)</t>
+          <t>A1c 손가락(少商·三間·前谷·商陽)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LU1</t>
+          <t>LI3, LU11, SI2, LI1</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1/1</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1/1</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1/1</t>
+          <t>0/4</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0/1</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
+          <t>0/4</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>0.536</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>D2 C7 극돌기(大椎)</t>
+          <t>A1a 수태음 본경 사슬(天府~太淵)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GB23</t>
+          <t>LU5, LU7, LU9, LU3, LU4, LU6, LU8</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1/1</t>
+          <t>7/7</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1/1</t>
+          <t>7/7</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>0/7</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0/1</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>0.584</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>A5 갈비활(期門)</t>
+          <t>A2a 앞가슴벽 2~5늑간</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>LR14</t>
+          <t>KI25, PC1, SP18, KI22, KI23, KI24, ST16, ST18</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1/1</t>
+          <t>8/8</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1/1</t>
+          <t>8/8</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>0/8</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0/1</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
+          <t>0/8</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>0.522</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>D2 C7 극돌기(大椎)</t>
+          <t>A2b 빗장 아래(俞府)</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -23661,12 +23739,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GV14</t>
+          <t>KI27</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>1/1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -23676,7 +23754,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>1/1</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -23689,7 +23767,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>D1 흉골 정중(玉堂)</t>
+          <t>A2c 앞가슴벽 바깥(中府)</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -23697,7 +23775,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CV18</t>
+          <t>LU1</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -23707,12 +23785,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>1/1</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>1/1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -23725,7 +23803,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>A4 명치(鳩尾)</t>
+          <t>A2d 옆가슴(輒筋)</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -23733,30 +23811,174 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>GB23</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>D 갈비활(期門)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>LR14</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>D C7 극돌기(大椎)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>GV14</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>D 흉골 정중(玉堂)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CV18</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>D 명치(鳩尾)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>CV15</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>0/1</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>0/1</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>0/1</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>0/1</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>